<commit_message>
Add feature analysis, imbalance study, charts and work split
- 04_feature_importance.py: permutation importance, redundant-feature
  detection, and the single features that best separate each attack from
  benign traffic. Results in results/features/.
- 05_imbalance.py: class weights, benign undersampling and SMOTE, applied
  to the training split only so the test scores stay honest.
- 06_charts.py + plot_style.py: report figures rendered from the results
  files, colour-blind-checked palette. results/charts/.
- common.py: one stratified sampler shared by every script.
- 03_kernel_pca.py: gamma tuning and repeat-sample seeds for stability;
  results reproduce the earlier run byte for byte.
- 02_experiment.py: test sizes 0.2/0.4/0.6, resumable, leaves cores free.
- docs/networking_background.md: the flow features and every attack in
  protocol terms, with the deployment discussion.
- WORK_SPLIT.md: who owns which track.
</commit_message>
<xml_diff>
--- a/results/kernel_pca/kpca_lr_s10000.xlsx
+++ b/results/kernel_pca/kpca_lr_s10000.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="accuracy" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="macro_f1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="all runs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="best per classifier" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kernel x classifier" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="all runs" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1069,12 +1071,168 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>classifier</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>baseline macro_f1 (mean of tests)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>best kernel</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>best gamma</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>best components</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>best test size</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>best macro_f1</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>best accuracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.4934</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.9367</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>classifier</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>rbf</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sigmoid</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cosine</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.3971</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.2012</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1803</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.2091</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>test_size</t>
         </is>
       </c>
@@ -1085,37 +1243,57 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>gamma_label</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>gamma</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>classifier</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>components</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sample_seed</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>n_train</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>n_test</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>macro_f1</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>seconds</t>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>clf_seconds</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>kpca_seconds</t>
         </is>
       </c>
     </row>
@@ -1130,26 +1308,38 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
         <v>8268</v>
       </c>
-      <c r="F2" t="n">
+      <c r="I2" t="n">
         <v>2068</v>
       </c>
-      <c r="G2" t="n">
+      <c r="J2" t="n">
         <v>0.956</v>
       </c>
-      <c r="H2" t="n">
+      <c r="K2" t="n">
         <v>0.6451</v>
       </c>
-      <c r="I2" t="n">
-        <v>0.4</v>
+      <c r="L2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1163,26 +1353,38 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
         <v>6201</v>
       </c>
-      <c r="F3" t="n">
+      <c r="I3" t="n">
         <v>4135</v>
       </c>
-      <c r="G3" t="n">
+      <c r="J3" t="n">
         <v>0.9453</v>
       </c>
-      <c r="H3" t="n">
+      <c r="K3" t="n">
         <v>0.6261</v>
       </c>
-      <c r="I3" t="n">
-        <v>0.3</v>
+      <c r="L3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1196,26 +1398,38 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
         <v>4134</v>
       </c>
-      <c r="F4" t="n">
+      <c r="I4" t="n">
         <v>6202</v>
       </c>
-      <c r="G4" t="n">
+      <c r="J4" t="n">
         <v>0.9442</v>
       </c>
-      <c r="H4" t="n">
+      <c r="K4" t="n">
         <v>0.5859</v>
       </c>
-      <c r="I4" t="n">
+      <c r="L4" t="n">
         <v>0.2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1229,26 +1443,38 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>8268</v>
       </c>
-      <c r="F5" t="n">
+      <c r="I5" t="n">
         <v>2068</v>
       </c>
-      <c r="G5" t="n">
+      <c r="J5" t="n">
         <v>0.8907</v>
       </c>
-      <c r="H5" t="n">
+      <c r="K5" t="n">
         <v>0.2785</v>
       </c>
-      <c r="I5" t="n">
-        <v>1.7</v>
+      <c r="L5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="6">
@@ -1262,26 +1488,38 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>5</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
         <v>6201</v>
       </c>
-      <c r="F6" t="n">
+      <c r="I6" t="n">
         <v>4135</v>
       </c>
-      <c r="G6" t="n">
+      <c r="J6" t="n">
         <v>0.8839</v>
       </c>
-      <c r="H6" t="n">
+      <c r="K6" t="n">
         <v>0.2639</v>
       </c>
-      <c r="I6" t="n">
-        <v>1.2</v>
+      <c r="L6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1295,26 +1533,38 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>5</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>4134</v>
       </c>
-      <c r="F7" t="n">
+      <c r="I7" t="n">
         <v>6202</v>
       </c>
-      <c r="G7" t="n">
+      <c r="J7" t="n">
         <v>0.8796</v>
       </c>
-      <c r="H7" t="n">
+      <c r="K7" t="n">
         <v>0.2689</v>
       </c>
-      <c r="I7" t="n">
-        <v>0.8</v>
+      <c r="L7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="8">
@@ -1328,26 +1578,40 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D8" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>5</v>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>8268</v>
       </c>
-      <c r="F8" t="n">
+      <c r="I8" t="n">
         <v>2068</v>
       </c>
-      <c r="G8" t="n">
+      <c r="J8" t="n">
         <v>0.8080000000000001</v>
       </c>
-      <c r="H8" t="n">
+      <c r="K8" t="n">
         <v>0.1542</v>
       </c>
-      <c r="I8" t="n">
-        <v>1.9</v>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="9">
@@ -1361,26 +1625,40 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>5</v>
       </c>
-      <c r="E9" t="n">
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>6201</v>
       </c>
-      <c r="F9" t="n">
+      <c r="I9" t="n">
         <v>4135</v>
       </c>
-      <c r="G9" t="n">
+      <c r="J9" t="n">
         <v>0.8073</v>
       </c>
-      <c r="H9" t="n">
+      <c r="K9" t="n">
         <v>0.1332</v>
       </c>
-      <c r="I9" t="n">
-        <v>1.7</v>
+      <c r="L9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1394,26 +1672,40 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D10" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
         <v>5</v>
       </c>
-      <c r="E10" t="n">
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
         <v>4134</v>
       </c>
-      <c r="F10" t="n">
+      <c r="I10" t="n">
         <v>6202</v>
       </c>
-      <c r="G10" t="n">
+      <c r="J10" t="n">
         <v>0.8088</v>
       </c>
-      <c r="H10" t="n">
+      <c r="K10" t="n">
         <v>0.1516</v>
       </c>
-      <c r="I10" t="n">
-        <v>0.9</v>
+      <c r="L10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="11">
@@ -1427,26 +1719,40 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D11" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
         <v>8268</v>
       </c>
-      <c r="F11" t="n">
+      <c r="I11" t="n">
         <v>2068</v>
       </c>
-      <c r="G11" t="n">
+      <c r="J11" t="n">
         <v>0.881</v>
       </c>
-      <c r="H11" t="n">
+      <c r="K11" t="n">
         <v>0.1569</v>
       </c>
-      <c r="I11" t="n">
-        <v>2</v>
+      <c r="L11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2.3</v>
       </c>
     </row>
     <row r="12">
@@ -1460,26 +1766,40 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D12" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>5</v>
       </c>
-      <c r="E12" t="n">
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
         <v>6201</v>
       </c>
-      <c r="F12" t="n">
+      <c r="I12" t="n">
         <v>4135</v>
       </c>
-      <c r="G12" t="n">
+      <c r="J12" t="n">
         <v>0.8767</v>
       </c>
-      <c r="H12" t="n">
+      <c r="K12" t="n">
         <v>0.153</v>
       </c>
-      <c r="I12" t="n">
-        <v>2</v>
+      <c r="L12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1.8</v>
       </c>
     </row>
     <row r="13">
@@ -1493,25 +1813,39 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D13" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>5</v>
       </c>
-      <c r="E13" t="n">
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
         <v>4134</v>
       </c>
-      <c r="F13" t="n">
+      <c r="I13" t="n">
         <v>6202</v>
       </c>
-      <c r="G13" t="n">
+      <c r="J13" t="n">
         <v>0.8783</v>
       </c>
-      <c r="H13" t="n">
+      <c r="K13" t="n">
         <v>0.1557</v>
       </c>
-      <c r="I13" t="n">
+      <c r="L13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1526,26 +1860,40 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D14" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>5</v>
       </c>
-      <c r="E14" t="n">
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
         <v>8268</v>
       </c>
-      <c r="F14" t="n">
+      <c r="I14" t="n">
         <v>2068</v>
       </c>
-      <c r="G14" t="n">
+      <c r="J14" t="n">
         <v>0.8781</v>
       </c>
-      <c r="H14" t="n">
+      <c r="K14" t="n">
         <v>0.1559</v>
       </c>
-      <c r="I14" t="n">
-        <v>1.5</v>
+      <c r="L14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1.3</v>
       </c>
     </row>
     <row r="15">
@@ -1559,25 +1907,39 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D15" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
         <v>5</v>
       </c>
-      <c r="E15" t="n">
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
         <v>6201</v>
       </c>
-      <c r="F15" t="n">
+      <c r="I15" t="n">
         <v>4135</v>
       </c>
-      <c r="G15" t="n">
+      <c r="J15" t="n">
         <v>0.8762</v>
       </c>
-      <c r="H15" t="n">
+      <c r="K15" t="n">
         <v>0.1533</v>
       </c>
-      <c r="I15" t="n">
+      <c r="L15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1592,25 +1954,39 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D16" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
         <v>5</v>
       </c>
-      <c r="E16" t="n">
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
         <v>4134</v>
       </c>
-      <c r="F16" t="n">
+      <c r="I16" t="n">
         <v>6202</v>
       </c>
-      <c r="G16" t="n">
+      <c r="J16" t="n">
         <v>0.8702</v>
       </c>
-      <c r="H16" t="n">
+      <c r="K16" t="n">
         <v>0.1473</v>
       </c>
-      <c r="I16" t="n">
+      <c r="L16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M16" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -1625,26 +2001,38 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>5</v>
       </c>
-      <c r="E17" t="n">
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
         <v>8268</v>
       </c>
-      <c r="F17" t="n">
+      <c r="I17" t="n">
         <v>2068</v>
       </c>
-      <c r="G17" t="n">
+      <c r="J17" t="n">
         <v>0.8912</v>
       </c>
-      <c r="H17" t="n">
+      <c r="K17" t="n">
         <v>0.1941</v>
       </c>
-      <c r="I17" t="n">
-        <v>1.1</v>
+      <c r="L17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1658,26 +2046,38 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>5</v>
       </c>
-      <c r="E18" t="n">
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
         <v>6201</v>
       </c>
-      <c r="F18" t="n">
+      <c r="I18" t="n">
         <v>4135</v>
       </c>
-      <c r="G18" t="n">
+      <c r="J18" t="n">
         <v>0.888</v>
       </c>
-      <c r="H18" t="n">
+      <c r="K18" t="n">
         <v>0.1883</v>
       </c>
-      <c r="I18" t="n">
-        <v>0.7</v>
+      <c r="L18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="19">
@@ -1691,26 +2091,38 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
         <v>5</v>
       </c>
-      <c r="E19" t="n">
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
         <v>4134</v>
       </c>
-      <c r="F19" t="n">
+      <c r="I19" t="n">
         <v>6202</v>
       </c>
-      <c r="G19" t="n">
+      <c r="J19" t="n">
         <v>0.8875</v>
       </c>
-      <c r="H19" t="n">
+      <c r="K19" t="n">
         <v>0.1892</v>
       </c>
-      <c r="I19" t="n">
-        <v>0.5</v>
+      <c r="L19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="20">
@@ -1724,26 +2136,38 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
         <v>10</v>
       </c>
-      <c r="E20" t="n">
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
         <v>8268</v>
       </c>
-      <c r="F20" t="n">
+      <c r="I20" t="n">
         <v>2068</v>
       </c>
-      <c r="G20" t="n">
+      <c r="J20" t="n">
         <v>0.9202</v>
       </c>
-      <c r="H20" t="n">
+      <c r="K20" t="n">
         <v>0.4496</v>
       </c>
-      <c r="I20" t="n">
-        <v>1.4</v>
+      <c r="L20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M20" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="21">
@@ -1757,26 +2181,38 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
         <v>10</v>
       </c>
-      <c r="E21" t="n">
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
         <v>6201</v>
       </c>
-      <c r="F21" t="n">
+      <c r="I21" t="n">
         <v>4135</v>
       </c>
-      <c r="G21" t="n">
+      <c r="J21" t="n">
         <v>0.9083</v>
       </c>
-      <c r="H21" t="n">
+      <c r="K21" t="n">
         <v>0.4307</v>
       </c>
-      <c r="I21" t="n">
-        <v>1.1</v>
+      <c r="L21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M21" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1790,26 +2226,38 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
         <v>10</v>
       </c>
-      <c r="E22" t="n">
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
         <v>4134</v>
       </c>
-      <c r="F22" t="n">
+      <c r="I22" t="n">
         <v>6202</v>
       </c>
-      <c r="G22" t="n">
+      <c r="J22" t="n">
         <v>0.9073</v>
       </c>
-      <c r="H22" t="n">
+      <c r="K22" t="n">
         <v>0.4218</v>
       </c>
-      <c r="I22" t="n">
-        <v>0.7</v>
+      <c r="L22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="23">
@@ -1823,26 +2271,40 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D23" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
         <v>10</v>
       </c>
-      <c r="E23" t="n">
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
         <v>8268</v>
       </c>
-      <c r="F23" t="n">
+      <c r="I23" t="n">
         <v>2068</v>
       </c>
-      <c r="G23" t="n">
+      <c r="J23" t="n">
         <v>0.8080000000000001</v>
       </c>
-      <c r="H23" t="n">
+      <c r="K23" t="n">
         <v>0.1415</v>
       </c>
-      <c r="I23" t="n">
-        <v>2.4</v>
+      <c r="L23" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M23" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="24">
@@ -1856,26 +2318,40 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D24" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
         <v>10</v>
       </c>
-      <c r="E24" t="n">
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
         <v>6201</v>
       </c>
-      <c r="F24" t="n">
+      <c r="I24" t="n">
         <v>4135</v>
       </c>
-      <c r="G24" t="n">
+      <c r="J24" t="n">
         <v>0.8094</v>
       </c>
-      <c r="H24" t="n">
+      <c r="K24" t="n">
         <v>0.1487</v>
       </c>
-      <c r="I24" t="n">
-        <v>2.1</v>
+      <c r="L24" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="25">
@@ -1889,26 +2365,40 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D25" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
         <v>10</v>
       </c>
-      <c r="E25" t="n">
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
         <v>4134</v>
       </c>
-      <c r="F25" t="n">
+      <c r="I25" t="n">
         <v>6202</v>
       </c>
-      <c r="G25" t="n">
+      <c r="J25" t="n">
         <v>0.8699</v>
       </c>
-      <c r="H25" t="n">
+      <c r="K25" t="n">
         <v>0.2383</v>
       </c>
-      <c r="I25" t="n">
-        <v>1</v>
+      <c r="L25" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="26">
@@ -1922,25 +2412,39 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D26" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
         <v>10</v>
       </c>
-      <c r="E26" t="n">
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
         <v>8268</v>
       </c>
-      <c r="F26" t="n">
+      <c r="I26" t="n">
         <v>2068</v>
       </c>
-      <c r="G26" t="n">
+      <c r="J26" t="n">
         <v>0.898</v>
       </c>
-      <c r="H26" t="n">
+      <c r="K26" t="n">
         <v>0.2008</v>
       </c>
-      <c r="I26" t="n">
+      <c r="L26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M26" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1955,26 +2459,40 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D27" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
         <v>10</v>
       </c>
-      <c r="E27" t="n">
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
         <v>6201</v>
       </c>
-      <c r="F27" t="n">
+      <c r="I27" t="n">
         <v>4135</v>
       </c>
-      <c r="G27" t="n">
+      <c r="J27" t="n">
         <v>0.8909</v>
       </c>
-      <c r="H27" t="n">
+      <c r="K27" t="n">
         <v>0.1919</v>
       </c>
-      <c r="I27" t="n">
-        <v>1.5</v>
+      <c r="L27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M27" t="n">
+        <v>1.6</v>
       </c>
     </row>
     <row r="28">
@@ -1988,26 +2506,40 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D28" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
         <v>10</v>
       </c>
-      <c r="E28" t="n">
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
         <v>4134</v>
       </c>
-      <c r="F28" t="n">
+      <c r="I28" t="n">
         <v>6202</v>
       </c>
-      <c r="G28" t="n">
+      <c r="J28" t="n">
         <v>0.8763</v>
       </c>
-      <c r="H28" t="n">
+      <c r="K28" t="n">
         <v>0.1543</v>
       </c>
-      <c r="I28" t="n">
-        <v>1</v>
+      <c r="L28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="29">
@@ -2021,25 +2553,39 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D29" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
         <v>10</v>
       </c>
-      <c r="E29" t="n">
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
         <v>8268</v>
       </c>
-      <c r="F29" t="n">
+      <c r="I29" t="n">
         <v>2068</v>
       </c>
-      <c r="G29" t="n">
+      <c r="J29" t="n">
         <v>0.9004</v>
       </c>
-      <c r="H29" t="n">
+      <c r="K29" t="n">
         <v>0.2057</v>
       </c>
-      <c r="I29" t="n">
+      <c r="L29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M29" t="n">
         <v>1.5</v>
       </c>
     </row>
@@ -2054,26 +2600,40 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D30" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
         <v>10</v>
       </c>
-      <c r="E30" t="n">
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
         <v>6201</v>
       </c>
-      <c r="F30" t="n">
+      <c r="I30" t="n">
         <v>4135</v>
       </c>
-      <c r="G30" t="n">
+      <c r="J30" t="n">
         <v>0.8909</v>
       </c>
-      <c r="H30" t="n">
+      <c r="K30" t="n">
         <v>0.1918</v>
       </c>
-      <c r="I30" t="n">
-        <v>1</v>
+      <c r="L30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M30" t="n">
+        <v>1.1</v>
       </c>
     </row>
     <row r="31">
@@ -2087,26 +2647,40 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D31" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
         <v>10</v>
       </c>
-      <c r="E31" t="n">
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
         <v>4134</v>
       </c>
-      <c r="F31" t="n">
+      <c r="I31" t="n">
         <v>6202</v>
       </c>
-      <c r="G31" t="n">
+      <c r="J31" t="n">
         <v>0.8862</v>
       </c>
-      <c r="H31" t="n">
+      <c r="K31" t="n">
         <v>0.1801</v>
       </c>
-      <c r="I31" t="n">
-        <v>0.6</v>
+      <c r="L31" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="32">
@@ -2120,25 +2694,37 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
         <v>10</v>
       </c>
-      <c r="E32" t="n">
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
         <v>8268</v>
       </c>
-      <c r="F32" t="n">
+      <c r="I32" t="n">
         <v>2068</v>
       </c>
-      <c r="G32" t="n">
+      <c r="J32" t="n">
         <v>0.9086</v>
       </c>
-      <c r="H32" t="n">
+      <c r="K32" t="n">
         <v>0.2206</v>
       </c>
-      <c r="I32" t="n">
+      <c r="L32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M32" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -2153,25 +2739,37 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
         <v>10</v>
       </c>
-      <c r="E33" t="n">
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
         <v>6201</v>
       </c>
-      <c r="F33" t="n">
+      <c r="I33" t="n">
         <v>4135</v>
       </c>
-      <c r="G33" t="n">
+      <c r="J33" t="n">
         <v>0.8999</v>
       </c>
-      <c r="H33" t="n">
+      <c r="K33" t="n">
         <v>0.2132</v>
       </c>
-      <c r="I33" t="n">
+      <c r="L33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M33" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -2186,25 +2784,37 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
         <v>10</v>
       </c>
-      <c r="E34" t="n">
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
         <v>4134</v>
       </c>
-      <c r="F34" t="n">
+      <c r="I34" t="n">
         <v>6202</v>
       </c>
-      <c r="G34" t="n">
+      <c r="J34" t="n">
         <v>0.8992</v>
       </c>
-      <c r="H34" t="n">
+      <c r="K34" t="n">
         <v>0.2088</v>
       </c>
-      <c r="I34" t="n">
+      <c r="L34" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M34" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -2219,26 +2829,38 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
         <v>15</v>
       </c>
-      <c r="E35" t="n">
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
         <v>8268</v>
       </c>
-      <c r="F35" t="n">
+      <c r="I35" t="n">
         <v>2068</v>
       </c>
-      <c r="G35" t="n">
+      <c r="J35" t="n">
         <v>0.9367</v>
       </c>
-      <c r="H35" t="n">
+      <c r="K35" t="n">
         <v>0.4934</v>
       </c>
-      <c r="I35" t="n">
-        <v>1.7</v>
+      <c r="L35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M35" t="n">
+        <v>1.3</v>
       </c>
     </row>
     <row r="36">
@@ -2252,26 +2874,38 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
         <v>15</v>
       </c>
-      <c r="E36" t="n">
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
         <v>6201</v>
       </c>
-      <c r="F36" t="n">
+      <c r="I36" t="n">
         <v>4135</v>
       </c>
-      <c r="G36" t="n">
+      <c r="J36" t="n">
         <v>0.9267</v>
       </c>
-      <c r="H36" t="n">
+      <c r="K36" t="n">
         <v>0.493</v>
       </c>
-      <c r="I36" t="n">
-        <v>1.5</v>
+      <c r="L36" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="37">
@@ -2285,26 +2919,38 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
         <v>15</v>
       </c>
-      <c r="E37" t="n">
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
         <v>4134</v>
       </c>
-      <c r="F37" t="n">
+      <c r="I37" t="n">
         <v>6202</v>
       </c>
-      <c r="G37" t="n">
+      <c r="J37" t="n">
         <v>0.9197</v>
       </c>
-      <c r="H37" t="n">
+      <c r="K37" t="n">
         <v>0.4744</v>
       </c>
-      <c r="I37" t="n">
-        <v>1.6</v>
+      <c r="L37" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="38">
@@ -2318,26 +2964,40 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D38" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
         <v>15</v>
       </c>
-      <c r="E38" t="n">
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
         <v>8268</v>
       </c>
-      <c r="F38" t="n">
+      <c r="I38" t="n">
         <v>2068</v>
       </c>
-      <c r="G38" t="n">
+      <c r="J38" t="n">
         <v>0.8796</v>
       </c>
-      <c r="H38" t="n">
+      <c r="K38" t="n">
         <v>0.2768</v>
       </c>
-      <c r="I38" t="n">
-        <v>3.8</v>
+      <c r="L38" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M38" t="n">
+        <v>1.3</v>
       </c>
     </row>
     <row r="39">
@@ -2351,26 +3011,40 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D39" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
         <v>15</v>
       </c>
-      <c r="E39" t="n">
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
         <v>6201</v>
       </c>
-      <c r="F39" t="n">
+      <c r="I39" t="n">
         <v>4135</v>
       </c>
-      <c r="G39" t="n">
+      <c r="J39" t="n">
         <v>0.8817</v>
       </c>
-      <c r="H39" t="n">
+      <c r="K39" t="n">
         <v>0.2809</v>
       </c>
-      <c r="I39" t="n">
-        <v>2.9</v>
+      <c r="L39" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M39" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -2384,26 +3058,40 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D40" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
         <v>15</v>
       </c>
-      <c r="E40" t="n">
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
         <v>4134</v>
       </c>
-      <c r="F40" t="n">
+      <c r="I40" t="n">
         <v>6202</v>
       </c>
-      <c r="G40" t="n">
+      <c r="J40" t="n">
         <v>0.8774999999999999</v>
       </c>
-      <c r="H40" t="n">
+      <c r="K40" t="n">
         <v>0.2856</v>
       </c>
-      <c r="I40" t="n">
-        <v>1.6</v>
+      <c r="L40" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="41">
@@ -2417,26 +3105,40 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D41" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
         <v>15</v>
       </c>
-      <c r="E41" t="n">
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
         <v>8268</v>
       </c>
-      <c r="F41" t="n">
+      <c r="I41" t="n">
         <v>2068</v>
       </c>
-      <c r="G41" t="n">
+      <c r="J41" t="n">
         <v>0.9091</v>
       </c>
-      <c r="H41" t="n">
+      <c r="K41" t="n">
         <v>0.2141</v>
       </c>
-      <c r="I41" t="n">
-        <v>3.2</v>
+      <c r="L41" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M41" t="n">
+        <v>2.3</v>
       </c>
     </row>
     <row r="42">
@@ -2450,26 +3152,40 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D42" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
         <v>15</v>
       </c>
-      <c r="E42" t="n">
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
         <v>6201</v>
       </c>
-      <c r="F42" t="n">
+      <c r="I42" t="n">
         <v>4135</v>
       </c>
-      <c r="G42" t="n">
+      <c r="J42" t="n">
         <v>0.8955</v>
       </c>
-      <c r="H42" t="n">
+      <c r="K42" t="n">
         <v>0.1961</v>
       </c>
-      <c r="I42" t="n">
-        <v>2.5</v>
+      <c r="L42" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M42" t="n">
+        <v>1.7</v>
       </c>
     </row>
     <row r="43">
@@ -2483,26 +3199,40 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D43" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
         <v>15</v>
       </c>
-      <c r="E43" t="n">
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
         <v>4134</v>
       </c>
-      <c r="F43" t="n">
+      <c r="I43" t="n">
         <v>6202</v>
       </c>
-      <c r="G43" t="n">
+      <c r="J43" t="n">
         <v>0.8957000000000001</v>
       </c>
-      <c r="H43" t="n">
+      <c r="K43" t="n">
         <v>0.2002</v>
       </c>
-      <c r="I43" t="n">
-        <v>1.6</v>
+      <c r="L43" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M43" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -2516,26 +3246,40 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D44" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
         <v>15</v>
       </c>
-      <c r="E44" t="n">
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
         <v>8268</v>
       </c>
-      <c r="F44" t="n">
+      <c r="I44" t="n">
         <v>2068</v>
       </c>
-      <c r="G44" t="n">
+      <c r="J44" t="n">
         <v>0.913</v>
       </c>
-      <c r="H44" t="n">
+      <c r="K44" t="n">
         <v>0.2965</v>
       </c>
-      <c r="I44" t="n">
-        <v>2.2</v>
+      <c r="L44" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M44" t="n">
+        <v>1.7</v>
       </c>
     </row>
     <row r="45">
@@ -2549,26 +3293,40 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D45" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
         <v>15</v>
       </c>
-      <c r="E45" t="n">
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
         <v>6201</v>
       </c>
-      <c r="F45" t="n">
+      <c r="I45" t="n">
         <v>4135</v>
       </c>
-      <c r="G45" t="n">
+      <c r="J45" t="n">
         <v>0.9013</v>
       </c>
-      <c r="H45" t="n">
+      <c r="K45" t="n">
         <v>0.253</v>
       </c>
-      <c r="I45" t="n">
-        <v>1.3</v>
+      <c r="L45" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M45" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="46">
@@ -2582,26 +3340,40 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D46" t="n">
+        <v>0.01449275362318841</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
         <v>15</v>
       </c>
-      <c r="E46" t="n">
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
         <v>4134</v>
       </c>
-      <c r="F46" t="n">
+      <c r="I46" t="n">
         <v>6202</v>
       </c>
-      <c r="G46" t="n">
+      <c r="J46" t="n">
         <v>0.8957000000000001</v>
       </c>
-      <c r="H46" t="n">
+      <c r="K46" t="n">
         <v>0.1981</v>
       </c>
-      <c r="I46" t="n">
-        <v>0.9</v>
+      <c r="L46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="47">
@@ -2615,26 +3387,38 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
         <v>15</v>
       </c>
-      <c r="E47" t="n">
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
         <v>8268</v>
       </c>
-      <c r="F47" t="n">
+      <c r="I47" t="n">
         <v>2068</v>
       </c>
-      <c r="G47" t="n">
+      <c r="J47" t="n">
         <v>0.9159</v>
       </c>
-      <c r="H47" t="n">
+      <c r="K47" t="n">
         <v>0.2293</v>
       </c>
-      <c r="I47" t="n">
-        <v>1.5</v>
+      <c r="L47" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M47" t="n">
+        <v>1.4</v>
       </c>
     </row>
     <row r="48">
@@ -2648,26 +3432,38 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
         <v>15</v>
       </c>
-      <c r="E48" t="n">
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
         <v>6201</v>
       </c>
-      <c r="F48" t="n">
+      <c r="I48" t="n">
         <v>4135</v>
       </c>
-      <c r="G48" t="n">
+      <c r="J48" t="n">
         <v>0.9067</v>
       </c>
-      <c r="H48" t="n">
+      <c r="K48" t="n">
         <v>0.2206</v>
       </c>
-      <c r="I48" t="n">
-        <v>1.2</v>
+      <c r="L48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M48" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -2681,26 +3477,38 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
         <v>15</v>
       </c>
-      <c r="E49" t="n">
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
         <v>4134</v>
       </c>
-      <c r="F49" t="n">
+      <c r="I49" t="n">
         <v>6202</v>
       </c>
-      <c r="G49" t="n">
+      <c r="J49" t="n">
         <v>0.9068000000000001</v>
       </c>
-      <c r="H49" t="n">
+      <c r="K49" t="n">
         <v>0.2175</v>
       </c>
-      <c r="I49" t="n">
-        <v>0.7</v>
+      <c r="L49" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>